<commit_message>
motor: superficie activable = min(derechos, ABRS); ABRS sin derecho pasa a reactivación opcional
- src/simulation.py: denominador y pago usan min(derechos, ABRS); nuevo parámetro ha_abrs_sin_derecho_reactivada repartido titular a titular por exceso; columna SUP_ACTIVABLE
- pages/2_Simulador.py: slider conectado, helpers consumen SUP_ACTIVABLE, textos reescritos
- scripts: VALID_300 nuevos anclajes; sup_adicional invoca con reactivación total + externas para preservar VALID_B = 159.302,93
- README.md: metodología reescrita
- Regenerados 8 Excel con motor corregido

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comparativa_300_todas_vs_500_menor65.xlsx
+++ b/comparativa_300_todas_vs_500_menor65.xlsx
@@ -545,13 +545,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>94487.59</v>
+        <v>87830.17999999999</v>
       </c>
       <c r="C10" t="n">
-        <v>84723.38</v>
+        <v>78823.94</v>
       </c>
       <c r="D10" t="n">
-        <v>9764.209999999999</v>
+        <v>9006.24</v>
       </c>
     </row>
     <row r="11">
@@ -561,13 +561,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>30734.97</v>
+        <v>27318</v>
       </c>
       <c r="C11" t="n">
-        <v>24016.02</v>
+        <v>21134.13</v>
       </c>
       <c r="D11" t="n">
-        <v>6718.95</v>
+        <v>6183.87</v>
       </c>
     </row>
     <row r="12">
@@ -577,13 +577,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>27781.65</v>
+        <v>23919.95</v>
       </c>
       <c r="C12" t="n">
-        <v>21331.04</v>
+        <v>18187.03</v>
       </c>
       <c r="D12" t="n">
-        <v>6450.61</v>
+        <v>5732.92</v>
       </c>
     </row>
     <row r="13">
@@ -593,13 +593,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>153004.21</v>
+        <v>139068.13</v>
       </c>
       <c r="C13" t="n">
-        <v>130070.44</v>
+        <v>118145.1</v>
       </c>
       <c r="D13" t="n">
-        <v>22933.77</v>
+        <v>20923.03</v>
       </c>
     </row>
     <row r="15">
@@ -638,13 +638,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>17229.99</v>
+        <v>17620.97</v>
       </c>
       <c r="C17" t="n">
-        <v>22483.58</v>
+        <v>23029.43</v>
       </c>
       <c r="D17" t="n">
-        <v>-5253.59</v>
+        <v>-5408.46</v>
       </c>
     </row>
     <row r="18">
@@ -654,13 +654,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3229.97</v>
+        <v>3158.57</v>
       </c>
       <c r="C18" t="n">
-        <v>5111.12</v>
+        <v>4951.79</v>
       </c>
       <c r="D18" t="n">
-        <v>-1881.15</v>
+        <v>-1793.22</v>
       </c>
     </row>
     <row r="19">
@@ -670,13 +670,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>3526.02</v>
+        <v>3340.12</v>
       </c>
       <c r="C19" t="n">
-        <v>5987.71</v>
+        <v>5620.48</v>
       </c>
       <c r="D19" t="n">
-        <v>-2461.69</v>
+        <v>-2280.36</v>
       </c>
     </row>
     <row r="20">

</xml_diff>